<commit_message>
Pooling calculator: use 4 ul of cfEpi_1 so its 4 nM dilution covers the pool aliquot
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118hMfJWJZ4DaiswK3vUJeT
</commit_message>
<xml_diff>
--- a/cfEpi_pooling_20261020.xlsx
+++ b/cfEpi_pooling_20261020.xlsx
@@ -376,7 +376,7 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Lowest molarity — barely above target</t>
+    <t xml:space="preserve">Molarity barely above target: 4 µl library used so ≥ 5 µl of 4 nM dilution is available</t>
   </si>
   <si>
     <t xml:space="preserve">Weighted ×1.5 (broad mark)</t>
@@ -1681,13 +1681,12 @@
       <c r="D12" s="10" t="n">
         <v>5.35</v>
       </c>
-      <c r="E12" s="4" t="n">
-        <f aca="false">$B$6</f>
-        <v>2</v>
+      <c r="E12" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="F12" s="11" t="n">
         <f aca="false">IF(D12&lt;=$B$5,0,E12*(D12/$B$5-1))</f>
-        <v>0.675</v>
+        <v>1.35</v>
       </c>
       <c r="G12" s="12" t="n">
         <f aca="false">D12*E12/(E12+F12)</f>

</xml_diff>